<commit_message>
Name both tools in the review workbook
</commit_message>
<xml_diff>
--- a/deliverables_geodb_datenquellen/Rueckmeldung_GeoLAB-Finder.xlsx
+++ b/deliverables_geodb_datenquellen/Rueckmeldung_GeoLAB-Finder.xlsx
@@ -472,7 +472,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Rückmeldung zu den GeoLAB-Findern</t>
+          <t>Rückmeldung zum GeoDB Geodata Index und zum SOEP Variable Finder</t>
         </is>
       </c>
     </row>
@@ -585,14 +585,14 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>GeoDB (Geodaten): https://geodb.geolab.soz.uni-bielefeld.de/</t>
+          <t>GeoDB Geodata Index (Geodaten): https://geodb.geolab.soz.uni-bielefeld.de/</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>SOEP-Variablen:   https://soep-faiss.geolab.soz.uni-bielefeld.de/</t>
+          <t>SOEP Variable Finder:            https://soep-faiss.geolab.soz.uni-bielefeld.de/</t>
         </is>
       </c>
     </row>

</xml_diff>